<commit_message>
Align OpenQuant product framing
</commit_message>
<xml_diff>
--- a/docs/openquant_scope_table.xlsx
+++ b/docs/openquant_scope_table.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exam Mapping'!$A$4:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'OpenQuant Coverage'!$A$4:$G$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Source Workbook'!$A$4:$C$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Missing Coverage'!$A$4:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Missing Coverage'!$A$4:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sources'!$A$4:$C$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Checks'!$A$4:$E$9</definedName>
   </definedNames>
@@ -7237,9 +7237,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -7249,7 +7249,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Implemented and tested, but not wired into current API/UI product flow</t>
+          <t>Wired into /analyse and shown in the model reliability panel</t>
         </is>
       </c>
     </row>
@@ -7274,9 +7274,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>Implemented/tested, but not wired into current API/UI product flow</t>
+          <t>Wired into /analyse and shown before detailed formula evidence</t>
         </is>
       </c>
     </row>
@@ -7311,9 +7311,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Implemented, but not wired into API/UI and not covered by dedicated tests</t>
+          <t>Wired into /analyse and UI; add dedicated tests next</t>
         </is>
       </c>
     </row>
@@ -7809,7 +7809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8175,101 +8175,69 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Implementation gap</t>
+          <t>Testing gap</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Assumption diagnostic wiring</t>
+          <t>Audit trail dedicated tests</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Implemented, not productized</t>
+          <t>Productized, not directly tested</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>DiagnosticBuilder exists and is tested but API/UI do not expose it</t>
+          <t>Audit trail is now returned by API/UI but lacks focused tests</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Call diagnostic builder in analysis flow and surface concise output in reliability/assumption panel</t>
+          <t>Add tests for audit payload shape and formula references</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Implementation gap</t>
+          <t>UX gap</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Audit trail wiring</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Implemented, not productized</t>
+          <t>Market-implied belief as first screen</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>AuditTrailBuilder exists but is not returned by API/UI and has no dedicated tests</t>
+          <t>README/strategy now say this, UI still includes fair-value framing</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Add API payload, UI disclosure panel, and tests before marking productized</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>UX gap</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Market-implied belief as first screen</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>README/strategy now say this, UI still includes fair-value framing</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
           <t>Move reverse DCF and assumptions before intrinsic-value verdict language</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F16"/>
+  <autoFilter ref="A4:F15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add companion teaching deck (51 cards) and update scope table
- companion.html: 51-card EPFL deck, H1-H4, full 1:1 with the final
  formula sheet; readability fixes (bar-label overlap, hero wrap on
  diversification/terminal, expvar band overflow) and on-grid defaults
  for fwdfut/optpayoff; all 51 formulas correctness-audited
- scope table: new 'Companion deck card' column mapping every formula
  to its card; Project Plan notes on the deck and its coverage

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/openquant_scope_table.xlsx
+++ b/docs/openquant_scope_table.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -751,7 +751,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Derivatives; bonds/rates lab; portfolio lab; project decision lab; full capital-structure policy lab.</t>
+          <t>Derivatives; bonds/rates lab; portfolio lab; project decision lab; full capital-structure policy lab. (These are now covered as teaching cards in the companion deck, though not yet as data-driven labs.)</t>
         </is>
       </c>
       <c r="C12" s="2" t="n"/>
@@ -772,6 +772,30 @@
       <c r="C13" s="2" t="n"/>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Companion deck</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Interactive teaching deck (frontend/public/companion.html): the EPFL Principles of Finance course as 51 cards (one idea, one visual, one live formula each). Distinct from the data-driven valuation lab. Published to GitHub Pages from the gh-pages branch as index.html (manual deploy, no CI).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Companion coverage</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>51 cards across H1-H4 give full 1:1 coverage of every formula on the EPFL final formula sheet. Per-formula mapping in Formula Inventory, column "Companion deck card". Updated 2026-06-24.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:B13"/>
@@ -2780,7 +2804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2794,6 +2818,7 @@
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2812,6 +2837,7 @@
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
+      <c r="L1" s="1" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -2829,6 +2855,7 @@
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
+      <c r="L2" s="3" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -2842,6 +2869,7 @@
       <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -2899,6 +2927,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Companion deck card</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -2956,6 +2989,11 @@
           <t>DCF discounting</t>
         </is>
       </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>pv</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -3013,6 +3051,11 @@
           <t>Used internally</t>
         </is>
       </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>pv (DF)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -3070,6 +3113,11 @@
           <t>No current product need</t>
         </is>
       </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>fv</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -3127,6 +3175,11 @@
           <t>Special case of growing perpetuity</t>
         </is>
       </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>perpetuity</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -3184,6 +3237,11 @@
           <t>Terminal value and DDM</t>
         </is>
       </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>growperp</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -3241,6 +3299,11 @@
           <t>Present in course/workbook; no reusable OpenQuant annuity function</t>
         </is>
       </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>annuity</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -3298,6 +3361,11 @@
           <t>Sample exam tested</t>
         </is>
       </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>growann</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -3355,6 +3423,11 @@
           <t>Bonds/Rates Lab</t>
         </is>
       </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>ear</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -3412,6 +3485,11 @@
           <t>Mainly rates/derivatives</t>
         </is>
       </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>contcomp</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -3469,6 +3547,11 @@
           <t>Bonds/Rates Lab</t>
         </is>
       </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>spot</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -3526,6 +3609,11 @@
           <t>Bonds/Rates Lab</t>
         </is>
       </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>forward</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -3583,6 +3671,11 @@
           <t>Bonds/Rates Lab</t>
         </is>
       </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>bond</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -3640,6 +3733,11 @@
           <t>Requires solver if productized</t>
         </is>
       </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>ytm</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -3697,6 +3795,11 @@
           <t>Bonds/Rates Lab</t>
         </is>
       </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
@@ -3754,6 +3857,11 @@
           <t>Bonds/Rates Lab</t>
         </is>
       </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -3811,6 +3919,11 @@
           <t>Verified in tests with pandas/numpy, but no reusable OpenQuant function</t>
         </is>
       </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>expvar</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
@@ -3868,6 +3981,11 @@
           <t>Verified in tests with pandas/numpy, but no reusable OpenQuant function</t>
         </is>
       </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>expvar</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -3925,6 +4043,11 @@
           <t>Volatility annualisation exists in core.utils; no standalone probability-law module</t>
         </is>
       </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>expvar</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
@@ -3982,6 +4105,11 @@
           <t>Used in beta estimation via Cov/Var, not a standalone product feature</t>
         </is>
       </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>covcorr</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
@@ -4039,6 +4167,11 @@
           <t>Used as an input in beta_from_correlation; no correlation-computation function</t>
         </is>
       </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>covcorr</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
@@ -4096,6 +4229,11 @@
           <t>Current product estimates beta from market price data</t>
         </is>
       </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -4153,6 +4291,11 @@
           <t>Exam 2 test; not current product input method</t>
         </is>
       </c>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
@@ -4210,6 +4353,11 @@
           <t>Computed directly in tests; no reusable product function</t>
         </is>
       </c>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>portvar</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -4267,6 +4415,11 @@
           <t>Computed directly in tests; min-variance helper exists separately</t>
         </is>
       </c>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>portvar</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
@@ -4324,6 +4477,11 @@
           <t>Formula sheet line; add in Portfolio Lab</t>
         </is>
       </c>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>portbeta</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
@@ -4381,6 +4539,11 @@
           <t>Implemented/tested; no product UI</t>
         </is>
       </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>minvar</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
@@ -4438,6 +4601,11 @@
           <t>Implemented/tested; Portfolio Lab</t>
         </is>
       </c>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>sharpe</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
@@ -4495,6 +4663,11 @@
           <t>Current product WACC cost of equity</t>
         </is>
       </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>capm</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
@@ -4552,6 +4725,11 @@
           <t>No standalone alpha implementation or product flow</t>
         </is>
       </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
@@ -4609,6 +4787,11 @@
           <t>Core current product</t>
         </is>
       </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>wacc</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
@@ -4666,6 +4849,11 @@
           <t>Implemented/tested, but not visible or used in current WACC output</t>
         </is>
       </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>hamada</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
@@ -4723,6 +4911,11 @@
           <t>Unlevering exists; full explicit relever-beta formula is not a separate implementation</t>
         </is>
       </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>hamada</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
@@ -4780,6 +4973,11 @@
           <t>Theory in course/exams, not an OpenQuant formula implementation</t>
         </is>
       </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="6" t="inlineStr">
@@ -4837,6 +5035,11 @@
           <t>Capital Structure Lab</t>
         </is>
       </c>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>mm2</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
@@ -4894,6 +5097,11 @@
           <t>PVTS exists, but full APV formula/workflow is not implemented</t>
         </is>
       </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>apv</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
@@ -4951,6 +5159,11 @@
           <t>Exam tested; not current UI</t>
         </is>
       </c>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>taxshield</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
@@ -5008,6 +5221,11 @@
           <t>Needed for full financing policy</t>
         </is>
       </c>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>distress</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
@@ -5065,6 +5283,11 @@
           <t>Core current product</t>
         </is>
       </c>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>fcf</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
@@ -5122,6 +5345,11 @@
           <t>Change in working capital can be used as input; explicit NWC component formula is not implemented</t>
         </is>
       </c>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>nwc</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
@@ -5179,6 +5407,11 @@
           <t>Core current product</t>
         </is>
       </c>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>terminal</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
@@ -5236,6 +5469,11 @@
           <t>Core current product</t>
         </is>
       </c>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>dcf</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
@@ -5293,6 +5531,11 @@
           <t>Core current product</t>
         </is>
       </c>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>—  (valuation lab only)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
@@ -5350,6 +5593,11 @@
           <t>Core current product</t>
         </is>
       </c>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>ddm</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
@@ -5407,6 +5655,11 @@
           <t>OpenQuant-specific practical layer</t>
         </is>
       </c>
+      <c r="L48" s="6" t="inlineStr">
+        <is>
+          <t>—  (valuation lab only)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
@@ -5464,6 +5717,11 @@
           <t>Implemented/tested; Project Lab missing</t>
         </is>
       </c>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>npv</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
@@ -5521,6 +5779,11 @@
           <t>Implemented/tested; Project Lab missing</t>
         </is>
       </c>
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>irr</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
@@ -5578,6 +5841,11 @@
           <t>Project Lab</t>
         </is>
       </c>
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>pi</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
@@ -5635,6 +5903,11 @@
           <t>DDM tests exist; not current product</t>
         </is>
       </c>
+      <c r="L52" s="6" t="inlineStr">
+        <is>
+          <t>ddm</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
@@ -5692,6 +5965,11 @@
           <t>DDM tests; not current product</t>
         </is>
       </c>
+      <c r="L53" s="6" t="inlineStr">
+        <is>
+          <t>ddm</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
@@ -5749,6 +6027,11 @@
           <t>Derivatives out of scope</t>
         </is>
       </c>
+      <c r="L54" s="6" t="inlineStr">
+        <is>
+          <t>fwdprice</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
@@ -5806,6 +6089,11 @@
           <t>Derivatives out of scope</t>
         </is>
       </c>
+      <c r="L55" s="6" t="inlineStr">
+        <is>
+          <t>putcall</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
@@ -5863,6 +6151,11 @@
           <t>Derivatives out of scope</t>
         </is>
       </c>
+      <c r="L56" s="6" t="inlineStr">
+        <is>
+          <t>optpayoff</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
@@ -5920,6 +6213,11 @@
           <t>Derivatives out of scope</t>
         </is>
       </c>
+      <c r="L57" s="6" t="inlineStr">
+        <is>
+          <t>binomial</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
@@ -5975,6 +6273,11 @@
       <c r="K58" s="6" t="inlineStr">
         <is>
           <t>Derivatives out of scope</t>
+        </is>
+      </c>
+      <c r="L58" s="6" t="inlineStr">
+        <is>
+          <t>bs</t>
         </is>
       </c>
     </row>

</xml_diff>